<commit_message>
feat: add lesson for creating a line chart in a spreadsheet with Python
</commit_message>
<xml_diff>
--- a/hello_03.xlsx
+++ b/hello_03.xlsx
@@ -142,18 +142,9 @@
         </rich>
       </tx>
     </title>
-    <view3D>
-      <rotX val="15"/>
-      <rotY val="20"/>
-      <rAngAx val="1"/>
-    </view3D>
-    <floor/>
-    <sideWall/>
-    <backWall/>
     <plotArea>
-      <bar3DChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -167,6 +158,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'New Worksheet'!$A$2:$A$10</f>
@@ -178,12 +177,9 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <gapDepth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
-        <axId val="1000"/>
-      </bar3DChart>
+      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -206,16 +202,6 @@
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
-      <serAx>
-        <axId val="1000"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </serAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>

</xml_diff>